<commit_message>
employer identity ladder: applicant fills the company sheet, the verifier checks what can be checked, scams are refused at import
- scripts/verify_employer.py: USCC check digit, sender domain, ICP number on the
  homepage, RDAP domain age (<180 days fails), Wayback first capture, public phone on
  the company's own page, footprint links; prints the manual steps and the sentence
  for the registry's verification field
- import_employer_roster.py: scam red flags refuse a row, apply_email must be on the
  company domain, --verification required
- SelfReportedEmployer.verification, tests refuse an empty one; 10 new tests
- the 岗位表 gains a 公司信息 sheet; employer page, claim templates and README stop
  calling a corporate email the verification

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/openhire-岗位表.xlsx
+++ b/docs/openhire-岗位表.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="岗位" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="公司信息" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="说明" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -58,7 +59,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -67,6 +68,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -524,97 +526,274 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>填写（示例请覆盖）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>公司全称</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>示例机器人（北京）有限公司</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>统一社会信用代码</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>91110000MA01ABCD2X</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>海外注册号及注册地（海外公司填）</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>官网域名</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>example-robotics.cn</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ICP 备案号（国内公司填）</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>京ICP备12345678号</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>官网上公开电话所在页面网址</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.example-robotics.cn/contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>公开电话</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>010-12345678</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>行业足迹链接一（产品页 / GitHub / 论文 / 报道）</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.example-robotics.cn/product</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>行业足迹链接二</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/example-robotics</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>经办人职务</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>招聘负责人</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>怎么填（两分钟）</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>1. 「岗位」这一页每行一个岗位，六列都用中文填，不用改格式。示例那一行删掉或覆盖都行。</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>2. 发布日期写岗位真正对外开放的那天，格式 2026-10-08。我们会按它算在架天数，并在数据里标明「雇主自报」。</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>3. 投递链接要是贵公司自己网站上的页面（https 开头）；没有的话写一个公司邮箱（如 hr@公司域名），不要写个人手机或微信。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>4. 薪资范围可以空着。写的话用 25k-40k/月 或 30万-50万/年 这种写法。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>5. 岗位描述把职责和要求直接粘进来即可，长短不限。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr"/>
+      <c r="A7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>怎么发</t>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>「公司信息」这一页：我们怎么核实，贵公司要给什么</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>用贵公司企业邮箱（公司域名的邮箱）把这个文件发到 gdchenhao@qq.com，主题写「岗位表 + 公司名」，正文留一个贵公司官网招聘页的网址。企业邮箱发出来本身就是身份核验，不需要营业执照。</t>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>企业邮箱只证明贵公司控制这个域名，证明不了公司真实存在，所以我们还会核：工商登记（按全称和统一社会信用代码查公示系统）、ICP 备案（域名绑到哪个法人）、域名年龄和网站历史、回拨官网上公开的电话、两个早于申请日的行业足迹。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>3 个工作日内上线或回信。免费，只读，不改排序，不卖任何东西。</t>
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>贵公司只要把这些信息填进「公司信息」页，核对由我们做，大多数自动完成，剩下的是查两个政府网站和打一个电话。海外公司填注册号和注册地，ICP 留空。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>我们核的是「公司存在且在智驾 / 具身 / AI 基础设施里」，不是替贵公司担保。每条岗位带「雇主自报」标记，一有举报先下架。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>90 天规则</t>
-        </is>
-      </c>
+      <c r="A12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
+          <t>怎么发</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>用贵公司企业邮箱（公司域名的邮箱）把这个文件发到 gdchenhao@qq.com，主题写「岗位表 + 公司名」，正文留一个贵公司官网招聘页的网址。企业邮箱发出来本身就是身份核验，不需要营业执照。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>3 个工作日内上线或回信。免费，只读，不改排序，不卖任何东西。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>90 天规则</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
           <t>每条岗位从发布日期起 90 天后自动下架。还在招的，把表再发一次就续上（发布日期不用改，我们按再次收到的日期续）。</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>不想继续了，发一封邮件说一声就全部下架。</t>
         </is>

</xml_diff>